<commit_message>
Update Patch/Wild Mon Docs
</commit_message>
<xml_diff>
--- a/Yellow Kaizo Patch and Important Documents/Wild Pokemon Encounters.xlsx
+++ b/Yellow Kaizo Patch and Important Documents/Wild Pokemon Encounters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Yellow Kaizo Patch and Important Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Yellow-Kaizo\Yellow Kaizo Patch and Important Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743010E1-4758-4865-823F-D56E0957B371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C00089B-2491-45B8-935E-5B80FD55444E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1955" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1985" uniqueCount="429">
   <si>
     <t>Location</t>
   </si>
@@ -4677,6 +4677,12 @@
   <si>
     <t xml:space="preserve"> Mansion</t>
   </si>
+  <si>
+    <t>Indigo Plateau</t>
+  </si>
+  <si>
+    <t>Mr Mime</t>
+  </si>
 </sst>
 </file>
 
@@ -4796,7 +4802,7 @@
       <name val="Helvetica Neue"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4837,6 +4843,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -4978,7 +4990,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -5431,11 +5443,20 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -20699,7 +20720,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>548</xdr:row>
+      <xdr:row>559</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20733,7 +20754,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>549</xdr:row>
+      <xdr:row>560</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20767,7 +20788,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>550</xdr:row>
+      <xdr:row>561</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20801,7 +20822,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>551</xdr:row>
+      <xdr:row>562</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20835,7 +20856,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>552</xdr:row>
+      <xdr:row>563</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20869,7 +20890,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>553</xdr:row>
+      <xdr:row>564</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20903,7 +20924,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>554</xdr:row>
+      <xdr:row>565</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20937,7 +20958,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>555</xdr:row>
+      <xdr:row>566</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -20971,7 +20992,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>556</xdr:row>
+      <xdr:row>567</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21005,7 +21026,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>559</xdr:row>
+      <xdr:row>570</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21039,7 +21060,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>560</xdr:row>
+      <xdr:row>571</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21073,7 +21094,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>561</xdr:row>
+      <xdr:row>572</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21107,7 +21128,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>562</xdr:row>
+      <xdr:row>573</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21141,7 +21162,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>563</xdr:row>
+      <xdr:row>574</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21175,7 +21196,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>564</xdr:row>
+      <xdr:row>575</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21209,7 +21230,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>565</xdr:row>
+      <xdr:row>576</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21243,7 +21264,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>566</xdr:row>
+      <xdr:row>577</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21277,7 +21298,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>567</xdr:row>
+      <xdr:row>578</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21311,7 +21332,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>570</xdr:row>
+      <xdr:row>581</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21345,7 +21366,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>571</xdr:row>
+      <xdr:row>582</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21379,7 +21400,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>572</xdr:row>
+      <xdr:row>583</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21413,7 +21434,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>573</xdr:row>
+      <xdr:row>584</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21447,7 +21468,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>574</xdr:row>
+      <xdr:row>585</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21481,7 +21502,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>575</xdr:row>
+      <xdr:row>586</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21515,7 +21536,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>576</xdr:row>
+      <xdr:row>587</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -21549,7 +21570,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>577</xdr:row>
+      <xdr:row>588</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -24609,7 +24630,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>557</xdr:row>
+      <xdr:row>568</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -24647,7 +24668,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>568</xdr:row>
+      <xdr:row>579</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -24685,7 +24706,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>579</xdr:row>
+      <xdr:row>590</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="342900" cy="342900"/>
@@ -24723,14 +24744,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>720184</xdr:colOff>
-      <xdr:row>578</xdr:row>
+      <xdr:row>589</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>116159</xdr:colOff>
-      <xdr:row>579</xdr:row>
-      <xdr:rowOff>29211</xdr:rowOff>
+      <xdr:row>590</xdr:row>
+      <xdr:rowOff>29212</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -24963,6 +24984,386 @@
     </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>548</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="image293.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5843A7F-EF0F-413A-B342-66740AA7664B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId113" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2777007" y="179157201"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>557</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="image310.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EAFECB3D-9832-4870-A6F6-423C58DE2EBA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId119" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2776189" y="185145091"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>556</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="image142.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6F3B5E0-5E03-41C1-8336-C01427BBD7B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId118" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2776189" y="184796616"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>555</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="image298.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3BFDA07-D29B-458D-8C9D-C18E844135F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId117" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2776189" y="184448140"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>553</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="image292.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FEA36EE3-3F15-4193-B214-88BF0D41059F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId116" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2776189" y="183751189"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>549</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="472" name="image322.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBFA5F4C-2F41-4497-B571-52F33C630440}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId137" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2777007" y="179499296"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>554</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="473" name="image52.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DB86D32-C79D-4CE1-9BB7-063B2C67ED6B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2779745" y="180391837"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>19439</xdr:colOff>
+      <xdr:row>551</xdr:row>
+      <xdr:rowOff>340178</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="474" name="image271.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C1A0629-4DEA-41BE-A0FD-32A1194F847B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId75" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2799184" y="179711479"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>551</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="476" name="image183.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9403123-B303-4D64-A2DD-B866E83F61CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId88" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2779745" y="179371301"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>550</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="342900" cy="342900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="486" name="image189.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2429CC06-E3B5-474D-8BDC-FE0331E15A08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId89" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2779745" y="179031122"/>
+          <a:ext cx="342900" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -25224,7 +25625,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N587"/>
+  <dimension ref="A1:N596"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -25338,7 +25739,7 @@
       <c r="L6" s="9"/>
     </row>
     <row r="7" spans="1:12" ht="27" customHeight="1">
-      <c r="A7" s="154" t="s">
+      <c r="A7" s="156" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="6"/>
@@ -25598,7 +25999,7 @@
       <c r="L20" s="9"/>
     </row>
     <row r="21" spans="1:12" ht="27" customHeight="1">
-      <c r="A21" s="154" t="s">
+      <c r="A21" s="156" t="s">
         <v>39</v>
       </c>
       <c r="B21" s="6"/>
@@ -25814,7 +26215,7 @@
       <c r="L31" s="9"/>
     </row>
     <row r="32" spans="1:12" ht="27" customHeight="1">
-      <c r="A32" s="154" t="s">
+      <c r="A32" s="156" t="s">
         <v>44</v>
       </c>
       <c r="B32" s="6"/>
@@ -26290,7 +26691,7 @@
       <c r="L56" s="43"/>
     </row>
     <row r="57" spans="1:12" ht="27" customHeight="1">
-      <c r="A57" s="154" t="s">
+      <c r="A57" s="156" t="s">
         <v>66</v>
       </c>
       <c r="B57" s="6"/>
@@ -26506,7 +26907,7 @@
       <c r="L67" s="9"/>
     </row>
     <row r="68" spans="1:12" ht="27" customHeight="1">
-      <c r="A68" s="154" t="s">
+      <c r="A68" s="156" t="s">
         <v>71</v>
       </c>
       <c r="B68" s="6"/>
@@ -27402,7 +27803,7 @@
       <c r="L113" s="9"/>
     </row>
     <row r="114" spans="1:12" ht="27" customHeight="1">
-      <c r="A114" s="154" t="s">
+      <c r="A114" s="156" t="s">
         <v>92</v>
       </c>
       <c r="B114" s="6"/>
@@ -27618,7 +28019,7 @@
       <c r="L124" s="9"/>
     </row>
     <row r="125" spans="1:12" ht="27" customHeight="1">
-      <c r="A125" s="154" t="s">
+      <c r="A125" s="156" t="s">
         <v>99</v>
       </c>
       <c r="B125" s="6"/>
@@ -27834,7 +28235,7 @@
       <c r="L135" s="9"/>
     </row>
     <row r="136" spans="1:12" ht="27" customHeight="1">
-      <c r="A136" s="154" t="s">
+      <c r="A136" s="156" t="s">
         <v>104</v>
       </c>
       <c r="B136" s="6"/>
@@ -28050,7 +28451,7 @@
       <c r="L146" s="9"/>
     </row>
     <row r="147" spans="1:12" ht="27" customHeight="1">
-      <c r="A147" s="154" t="s">
+      <c r="A147" s="156" t="s">
         <v>109</v>
       </c>
       <c r="B147" s="6"/>
@@ -28392,7 +28793,7 @@
       <c r="L161" s="9"/>
     </row>
     <row r="162" spans="1:12" ht="27" customHeight="1">
-      <c r="A162" s="154" t="s">
+      <c r="A162" s="156" t="s">
         <v>119</v>
       </c>
       <c r="B162" s="6"/>
@@ -28608,7 +29009,7 @@
       <c r="L172" s="9"/>
     </row>
     <row r="173" spans="1:12" ht="27" customHeight="1">
-      <c r="A173" s="154" t="s">
+      <c r="A173" s="156" t="s">
         <v>121</v>
       </c>
       <c r="B173" s="6"/>
@@ -28824,7 +29225,7 @@
       <c r="L183" s="9"/>
     </row>
     <row r="184" spans="1:12" ht="27" customHeight="1">
-      <c r="A184" s="154" t="s">
+      <c r="A184" s="156" t="s">
         <v>126</v>
       </c>
       <c r="B184" s="6"/>
@@ -29728,7 +30129,7 @@
       <c r="L230" s="9"/>
     </row>
     <row r="231" spans="1:12" ht="27" customHeight="1">
-      <c r="A231" s="154" t="s">
+      <c r="A231" s="156" t="s">
         <v>159</v>
       </c>
       <c r="B231" s="6"/>
@@ -29944,7 +30345,7 @@
       <c r="L241" s="9"/>
     </row>
     <row r="242" spans="1:12" ht="27" customHeight="1">
-      <c r="A242" s="154" t="s">
+      <c r="A242" s="156" t="s">
         <v>161</v>
       </c>
       <c r="B242" s="6"/>
@@ -30204,7 +30605,7 @@
       <c r="L255" s="9"/>
     </row>
     <row r="256" spans="1:12" ht="27" customHeight="1">
-      <c r="A256" s="154" t="s">
+      <c r="A256" s="156" t="s">
         <v>169</v>
       </c>
       <c r="B256" s="6"/>
@@ -30481,7 +30882,7 @@
       <c r="L266" s="9"/>
     </row>
     <row r="267" spans="1:14" ht="27" customHeight="1">
-      <c r="A267" s="154" t="s">
+      <c r="A267" s="156" t="s">
         <v>176</v>
       </c>
       <c r="B267" s="6"/>
@@ -30757,7 +31158,7 @@
       <c r="L277" s="9"/>
     </row>
     <row r="278" spans="1:12" ht="27" customHeight="1">
-      <c r="A278" s="154" t="s">
+      <c r="A278" s="156" t="s">
         <v>179</v>
       </c>
       <c r="B278" s="6"/>
@@ -30973,7 +31374,7 @@
       <c r="L288" s="9"/>
     </row>
     <row r="289" spans="1:12" ht="27" customHeight="1">
-      <c r="A289" s="154" t="s">
+      <c r="A289" s="156" t="s">
         <v>185</v>
       </c>
       <c r="B289" s="6"/>
@@ -31392,7 +31793,7 @@
     </row>
     <row r="311" spans="1:12" ht="27" customHeight="1">
       <c r="A311" s="5"/>
-      <c r="B311" s="156" t="s">
+      <c r="B311" s="154" t="s">
         <v>200</v>
       </c>
       <c r="C311" s="15"/>
@@ -31588,7 +31989,7 @@
     </row>
     <row r="321" spans="1:12" ht="27" customHeight="1">
       <c r="A321" s="5"/>
-      <c r="B321" s="156" t="s">
+      <c r="B321" s="154" t="s">
         <v>209</v>
       </c>
       <c r="C321" s="15"/>
@@ -31804,7 +32205,7 @@
     </row>
     <row r="332" spans="1:12" ht="27" customHeight="1">
       <c r="A332" s="5"/>
-      <c r="B332" s="156" t="s">
+      <c r="B332" s="154" t="s">
         <v>211</v>
       </c>
       <c r="C332" s="15"/>
@@ -31999,7 +32400,7 @@
       <c r="L341" s="9"/>
     </row>
     <row r="342" spans="1:12" ht="27" customHeight="1">
-      <c r="A342" s="154" t="s">
+      <c r="A342" s="156" t="s">
         <v>213</v>
       </c>
       <c r="B342" s="6"/>
@@ -32215,7 +32616,7 @@
       <c r="L352" s="9"/>
     </row>
     <row r="353" spans="1:12" ht="27" customHeight="1">
-      <c r="A353" s="154" t="s">
+      <c r="A353" s="156" t="s">
         <v>218</v>
       </c>
       <c r="B353" s="6"/>
@@ -32431,7 +32832,7 @@
       <c r="L363" s="9"/>
     </row>
     <row r="364" spans="1:12" ht="27" customHeight="1">
-      <c r="A364" s="154" t="s">
+      <c r="A364" s="156" t="s">
         <v>220</v>
       </c>
       <c r="B364" s="6"/>
@@ -32801,7 +33202,7 @@
       <c r="L383" s="9"/>
     </row>
     <row r="384" spans="1:12" ht="27" customHeight="1">
-      <c r="A384" s="154" t="s">
+      <c r="A384" s="156" t="s">
         <v>227</v>
       </c>
       <c r="B384" s="6"/>
@@ -32977,7 +33378,7 @@
       <c r="L392" s="9"/>
     </row>
     <row r="393" spans="1:12" ht="27" customHeight="1">
-      <c r="A393" s="154" t="s">
+      <c r="A393" s="156" t="s">
         <v>231</v>
       </c>
       <c r="B393" s="6"/>
@@ -35087,7 +35488,7 @@
       <c r="L495" s="9"/>
     </row>
     <row r="496" spans="1:12" ht="27" customHeight="1">
-      <c r="A496" s="154" t="s">
+      <c r="A496" s="156" t="s">
         <v>258</v>
       </c>
       <c r="B496" s="6"/>
@@ -35331,7 +35732,7 @@
       <c r="L505" s="9"/>
     </row>
     <row r="506" spans="1:12" ht="27" customHeight="1">
-      <c r="A506" s="154" t="s">
+      <c r="A506" s="156" t="s">
         <v>263</v>
       </c>
       <c r="B506" s="6"/>
@@ -36162,249 +36563,249 @@
       <c r="K547" s="19"/>
       <c r="L547" s="19"/>
     </row>
-    <row r="548" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A548" s="92"/>
-      <c r="B548" s="93"/>
-      <c r="C548" s="94"/>
-      <c r="D548" s="95"/>
-      <c r="E548" s="94"/>
-      <c r="F548" s="94"/>
-      <c r="G548" s="94"/>
-      <c r="H548" s="94"/>
-      <c r="I548" s="95"/>
-      <c r="J548" s="94"/>
-      <c r="K548" s="94"/>
-      <c r="L548" s="94"/>
+    <row r="548" spans="1:12" ht="22.5" customHeight="1">
+      <c r="A548" s="5"/>
+      <c r="B548" s="6"/>
+      <c r="C548" s="157"/>
+      <c r="D548" s="158"/>
+      <c r="E548" s="157"/>
+      <c r="F548" s="157"/>
+      <c r="G548" s="157"/>
+      <c r="H548" s="157"/>
+      <c r="I548" s="158"/>
+      <c r="J548" s="157"/>
+      <c r="K548" s="157"/>
+      <c r="L548" s="157"/>
     </row>
     <row r="549" spans="1:12" ht="27" customHeight="1">
-      <c r="A549" s="96" t="s">
-        <v>279</v>
-      </c>
-      <c r="B549" s="97" t="s">
-        <v>81</v>
-      </c>
-      <c r="C549" s="98"/>
-      <c r="D549" s="99" t="s">
+      <c r="A549" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="B549" s="6"/>
+      <c r="C549" s="157"/>
+      <c r="D549" s="158" t="s">
         <v>21</v>
       </c>
-      <c r="E549" s="98" t="s">
-        <v>280</v>
-      </c>
-      <c r="F549" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G549" s="98"/>
-      <c r="H549" s="98"/>
-      <c r="I549" s="99"/>
-      <c r="J549" s="98"/>
-      <c r="K549" s="98"/>
-      <c r="L549" s="98"/>
+      <c r="E549" s="157" t="s">
+        <v>264</v>
+      </c>
+      <c r="F549" s="157" t="s">
+        <v>265</v>
+      </c>
+      <c r="G549" s="157"/>
+      <c r="H549" s="157"/>
+      <c r="I549" s="158"/>
+      <c r="J549" s="157"/>
+      <c r="K549" s="157"/>
+      <c r="L549" s="157"/>
     </row>
     <row r="550" spans="1:12" ht="27" customHeight="1">
-      <c r="A550" s="92"/>
-      <c r="B550" s="93"/>
-      <c r="C550" s="98"/>
-      <c r="D550" s="99" t="s">
+      <c r="A550" s="5"/>
+      <c r="B550" s="6"/>
+      <c r="C550" s="157"/>
+      <c r="D550" s="158" t="s">
         <v>24</v>
       </c>
-      <c r="E550" s="98" t="s">
-        <v>281</v>
-      </c>
-      <c r="F550" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G550" s="98"/>
-      <c r="H550" s="98"/>
-      <c r="I550" s="99"/>
-      <c r="J550" s="98"/>
-      <c r="K550" s="98"/>
-      <c r="L550" s="98"/>
+      <c r="E550" s="157" t="s">
+        <v>288</v>
+      </c>
+      <c r="F550" s="157" t="s">
+        <v>75</v>
+      </c>
+      <c r="G550" s="157"/>
+      <c r="H550" s="157"/>
+      <c r="I550" s="158"/>
+      <c r="J550" s="157"/>
+      <c r="K550" s="157"/>
+      <c r="L550" s="157"/>
     </row>
     <row r="551" spans="1:12" ht="27" customHeight="1">
-      <c r="A551" s="92"/>
-      <c r="B551" s="93"/>
-      <c r="C551" s="98"/>
-      <c r="D551" s="99" t="s">
+      <c r="A551" s="5"/>
+      <c r="B551" s="6"/>
+      <c r="C551" s="157"/>
+      <c r="D551" s="158" t="s">
         <v>24</v>
       </c>
-      <c r="E551" s="98" t="s">
-        <v>282</v>
-      </c>
-      <c r="F551" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G551" s="98"/>
-      <c r="H551" s="98"/>
-      <c r="I551" s="99"/>
-      <c r="J551" s="98"/>
-      <c r="K551" s="98"/>
-      <c r="L551" s="98"/>
+      <c r="E551" s="157" t="s">
+        <v>208</v>
+      </c>
+      <c r="F551" s="157" t="s">
+        <v>75</v>
+      </c>
+      <c r="G551" s="157"/>
+      <c r="H551" s="157"/>
+      <c r="I551" s="158"/>
+      <c r="J551" s="157"/>
+      <c r="K551" s="157"/>
+      <c r="L551" s="157"/>
     </row>
     <row r="552" spans="1:12" ht="27" customHeight="1">
-      <c r="A552" s="92"/>
-      <c r="B552" s="93"/>
-      <c r="C552" s="98"/>
-      <c r="D552" s="99" t="s">
+      <c r="A552" s="5"/>
+      <c r="B552" s="6"/>
+      <c r="C552" s="157"/>
+      <c r="D552" s="158" t="s">
         <v>27</v>
       </c>
-      <c r="E552" s="98" t="s">
-        <v>273</v>
-      </c>
-      <c r="F552" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G552" s="98"/>
-      <c r="H552" s="98"/>
-      <c r="I552" s="99"/>
-      <c r="J552" s="98"/>
-      <c r="K552" s="98"/>
-      <c r="L552" s="98"/>
+      <c r="E552" s="157" t="s">
+        <v>206</v>
+      </c>
+      <c r="F552" s="157" t="s">
+        <v>265</v>
+      </c>
+      <c r="G552" s="157"/>
+      <c r="H552" s="157"/>
+      <c r="I552" s="158"/>
+      <c r="J552" s="157"/>
+      <c r="K552" s="157"/>
+      <c r="L552" s="157"/>
     </row>
     <row r="553" spans="1:12" ht="27" customHeight="1">
-      <c r="A553" s="92"/>
-      <c r="B553" s="93"/>
-      <c r="C553" s="11"/>
-      <c r="D553" s="99" t="s">
+      <c r="A553" s="159"/>
+      <c r="B553" s="6"/>
+      <c r="C553" s="157"/>
+      <c r="D553" s="158" t="s">
         <v>27</v>
       </c>
-      <c r="E553" s="98" t="s">
+      <c r="E553" s="157" t="s">
+        <v>183</v>
+      </c>
+      <c r="F553" s="157" t="s">
+        <v>75</v>
+      </c>
+      <c r="G553" s="157"/>
+      <c r="H553" s="157"/>
+      <c r="I553" s="158"/>
+      <c r="J553" s="157"/>
+      <c r="K553" s="157"/>
+      <c r="L553" s="157"/>
+    </row>
+    <row r="554" spans="1:12" ht="27" customHeight="1">
+      <c r="A554" s="5"/>
+      <c r="B554" s="6"/>
+      <c r="C554" s="157"/>
+      <c r="D554" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="E554" s="157" t="s">
+        <v>268</v>
+      </c>
+      <c r="F554" s="157" t="s">
+        <v>261</v>
+      </c>
+      <c r="G554" s="157"/>
+      <c r="H554" s="157"/>
+      <c r="I554" s="158"/>
+      <c r="J554" s="157"/>
+      <c r="K554" s="157"/>
+      <c r="L554" s="157"/>
+    </row>
+    <row r="555" spans="1:12" ht="27" customHeight="1">
+      <c r="A555" s="5"/>
+      <c r="B555" s="6"/>
+      <c r="C555" s="157"/>
+      <c r="D555" s="158" t="s">
+        <v>31</v>
+      </c>
+      <c r="E555" s="157" t="s">
+        <v>428</v>
+      </c>
+      <c r="F555" s="157" t="s">
+        <v>261</v>
+      </c>
+      <c r="G555" s="157"/>
+      <c r="H555" s="157"/>
+      <c r="I555" s="158"/>
+      <c r="J555" s="157"/>
+      <c r="K555" s="157"/>
+      <c r="L555" s="157"/>
+    </row>
+    <row r="556" spans="1:12" ht="27" customHeight="1">
+      <c r="A556" s="5"/>
+      <c r="B556" s="6"/>
+      <c r="C556" s="157"/>
+      <c r="D556" s="158" t="s">
+        <v>31</v>
+      </c>
+      <c r="E556" s="157" t="s">
+        <v>269</v>
+      </c>
+      <c r="F556" s="157" t="s">
+        <v>270</v>
+      </c>
+      <c r="G556" s="157"/>
+      <c r="H556" s="157"/>
+      <c r="I556" s="158"/>
+      <c r="J556" s="157"/>
+      <c r="K556" s="157"/>
+      <c r="L556" s="157"/>
+    </row>
+    <row r="557" spans="1:12" ht="27" customHeight="1">
+      <c r="A557" s="5"/>
+      <c r="B557" s="6"/>
+      <c r="C557" s="157"/>
+      <c r="D557" s="158" t="s">
+        <v>51</v>
+      </c>
+      <c r="E557" s="157" t="s">
         <v>189</v>
       </c>
-      <c r="F553" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G553" s="98"/>
-      <c r="H553" s="98"/>
-      <c r="I553" s="99"/>
-      <c r="J553" s="98"/>
-      <c r="K553" s="98"/>
-      <c r="L553" s="98"/>
-    </row>
-    <row r="554" spans="1:12" ht="27" customHeight="1">
-      <c r="A554" s="92"/>
-      <c r="B554" s="93"/>
-      <c r="C554" s="98"/>
-      <c r="D554" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E554" s="98" t="s">
-        <v>283</v>
-      </c>
-      <c r="F554" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G554" s="98"/>
-      <c r="H554" s="98"/>
-      <c r="I554" s="99"/>
-      <c r="J554" s="98"/>
-      <c r="K554" s="98"/>
-      <c r="L554" s="98"/>
-    </row>
-    <row r="555" spans="1:12" ht="27" customHeight="1">
-      <c r="A555" s="92"/>
-      <c r="B555" s="93"/>
-      <c r="C555" s="98"/>
-      <c r="D555" s="99" t="s">
-        <v>31</v>
-      </c>
-      <c r="E555" s="98" t="s">
-        <v>208</v>
-      </c>
-      <c r="F555" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G555" s="98"/>
-      <c r="H555" s="98"/>
-      <c r="I555" s="99"/>
-      <c r="J555" s="98"/>
-      <c r="K555" s="98"/>
-      <c r="L555" s="98"/>
-    </row>
-    <row r="556" spans="1:12" ht="27" customHeight="1">
-      <c r="A556" s="92"/>
-      <c r="B556" s="93"/>
-      <c r="C556" s="98"/>
-      <c r="D556" s="99" t="s">
-        <v>31</v>
-      </c>
-      <c r="E556" s="98" t="s">
-        <v>284</v>
-      </c>
-      <c r="F556" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G556" s="98"/>
-      <c r="H556" s="98"/>
-      <c r="I556" s="99"/>
-      <c r="J556" s="98"/>
-      <c r="K556" s="98"/>
-      <c r="L556" s="98"/>
-    </row>
-    <row r="557" spans="1:12" ht="27" customHeight="1">
-      <c r="A557" s="92"/>
-      <c r="B557" s="93"/>
-      <c r="C557" s="98"/>
-      <c r="D557" s="99" t="s">
-        <v>51</v>
-      </c>
-      <c r="E557" s="98" t="s">
-        <v>285</v>
-      </c>
-      <c r="F557" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G557" s="98"/>
-      <c r="H557" s="98"/>
-      <c r="I557" s="99"/>
-      <c r="J557" s="98"/>
-      <c r="K557" s="98"/>
-      <c r="L557" s="98"/>
+      <c r="F557" s="157" t="s">
+        <v>261</v>
+      </c>
+      <c r="G557" s="157"/>
+      <c r="H557" s="157"/>
+      <c r="I557" s="158"/>
+      <c r="J557" s="157"/>
+      <c r="K557" s="157"/>
+      <c r="L557" s="157"/>
     </row>
     <row r="558" spans="1:12" ht="27" customHeight="1">
-      <c r="A558" s="92"/>
-      <c r="B558" s="93"/>
-      <c r="C558" s="98"/>
-      <c r="D558" s="99" t="s">
+      <c r="A558" s="5"/>
+      <c r="B558" s="6"/>
+      <c r="C558" s="157"/>
+      <c r="D558" s="158" t="s">
         <v>36</v>
       </c>
-      <c r="E558" s="98" t="s">
-        <v>15</v>
-      </c>
-      <c r="F558" s="98" t="s">
-        <v>228</v>
-      </c>
-      <c r="G558" s="98"/>
-      <c r="H558" s="98"/>
-      <c r="I558" s="99"/>
-      <c r="J558" s="98"/>
-      <c r="K558" s="98"/>
-      <c r="L558" s="98"/>
+      <c r="E558" s="157" t="s">
+        <v>271</v>
+      </c>
+      <c r="F558" s="157" t="s">
+        <v>270</v>
+      </c>
+      <c r="G558" s="157"/>
+      <c r="H558" s="157"/>
+      <c r="I558" s="158"/>
+      <c r="J558" s="157"/>
+      <c r="K558" s="157"/>
+      <c r="L558" s="157"/>
     </row>
     <row r="559" spans="1:12" ht="15.75" customHeight="1">
       <c r="A559" s="92"/>
       <c r="B559" s="93"/>
-      <c r="C559" s="98"/>
-      <c r="D559" s="99"/>
-      <c r="E559" s="98"/>
-      <c r="F559" s="98"/>
-      <c r="G559" s="98"/>
-      <c r="H559" s="98"/>
-      <c r="I559" s="99"/>
-      <c r="J559" s="98"/>
-      <c r="K559" s="98"/>
-      <c r="L559" s="98"/>
+      <c r="C559" s="94"/>
+      <c r="D559" s="95"/>
+      <c r="E559" s="94"/>
+      <c r="F559" s="94"/>
+      <c r="G559" s="94"/>
+      <c r="H559" s="94"/>
+      <c r="I559" s="95"/>
+      <c r="J559" s="94"/>
+      <c r="K559" s="94"/>
+      <c r="L559" s="94"/>
     </row>
     <row r="560" spans="1:12" ht="27" customHeight="1">
-      <c r="A560" s="92"/>
+      <c r="A560" s="96" t="s">
+        <v>279</v>
+      </c>
       <c r="B560" s="97" t="s">
-        <v>141</v>
+        <v>81</v>
       </c>
       <c r="C560" s="98"/>
       <c r="D560" s="99" t="s">
         <v>21</v>
       </c>
       <c r="E560" s="98" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="F560" s="98" t="s">
         <v>228</v>
@@ -36444,7 +36845,7 @@
         <v>24</v>
       </c>
       <c r="E562" s="98" t="s">
-        <v>251</v>
+        <v>282</v>
       </c>
       <c r="F562" s="98" t="s">
         <v>228</v>
@@ -36464,7 +36865,7 @@
         <v>27</v>
       </c>
       <c r="E563" s="98" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="F563" s="98" t="s">
         <v>228</v>
@@ -36479,12 +36880,12 @@
     <row r="564" spans="1:12" ht="27" customHeight="1">
       <c r="A564" s="92"/>
       <c r="B564" s="93"/>
-      <c r="C564" s="98"/>
+      <c r="C564" s="11"/>
       <c r="D564" s="99" t="s">
         <v>27</v>
       </c>
       <c r="E564" s="98" t="s">
-        <v>276</v>
+        <v>189</v>
       </c>
       <c r="F564" s="98" t="s">
         <v>228</v>
@@ -36504,7 +36905,7 @@
         <v>27</v>
       </c>
       <c r="E565" s="98" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F565" s="98" t="s">
         <v>228</v>
@@ -36524,7 +36925,7 @@
         <v>31</v>
       </c>
       <c r="E566" s="98" t="s">
-        <v>288</v>
+        <v>208</v>
       </c>
       <c r="F566" s="98" t="s">
         <v>228</v>
@@ -36544,7 +36945,7 @@
         <v>31</v>
       </c>
       <c r="E567" s="98" t="s">
-        <v>206</v>
+        <v>284</v>
       </c>
       <c r="F567" s="98" t="s">
         <v>228</v>
@@ -36559,12 +36960,12 @@
     <row r="568" spans="1:12" ht="27" customHeight="1">
       <c r="A568" s="92"/>
       <c r="B568" s="93"/>
-      <c r="C568" s="11"/>
+      <c r="C568" s="98"/>
       <c r="D568" s="99" t="s">
         <v>51</v>
       </c>
       <c r="E568" s="98" t="s">
-        <v>15</v>
+        <v>285</v>
       </c>
       <c r="F568" s="98" t="s">
         <v>228</v>
@@ -36584,7 +36985,7 @@
         <v>36</v>
       </c>
       <c r="E569" s="98" t="s">
-        <v>171</v>
+        <v>15</v>
       </c>
       <c r="F569" s="98" t="s">
         <v>228</v>
@@ -36613,14 +37014,14 @@
     <row r="571" spans="1:12" ht="27" customHeight="1">
       <c r="A571" s="92"/>
       <c r="B571" s="97" t="s">
-        <v>86</v>
+        <v>141</v>
       </c>
       <c r="C571" s="98"/>
       <c r="D571" s="99" t="s">
         <v>21</v>
       </c>
       <c r="E571" s="98" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="F571" s="98" t="s">
         <v>228</v>
@@ -36640,7 +37041,7 @@
         <v>24</v>
       </c>
       <c r="E572" s="98" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="F572" s="98" t="s">
         <v>228</v>
@@ -36660,7 +37061,7 @@
         <v>24</v>
       </c>
       <c r="E573" s="98" t="s">
-        <v>290</v>
+        <v>251</v>
       </c>
       <c r="F573" s="98" t="s">
         <v>228</v>
@@ -36680,7 +37081,7 @@
         <v>27</v>
       </c>
       <c r="E574" s="98" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="F574" s="98" t="s">
         <v>228</v>
@@ -36700,7 +37101,7 @@
         <v>27</v>
       </c>
       <c r="E575" s="98" t="s">
-        <v>219</v>
+        <v>276</v>
       </c>
       <c r="F575" s="98" t="s">
         <v>228</v>
@@ -36720,7 +37121,7 @@
         <v>27</v>
       </c>
       <c r="E576" s="98" t="s">
-        <v>226</v>
+        <v>287</v>
       </c>
       <c r="F576" s="98" t="s">
         <v>228</v>
@@ -36740,7 +37141,7 @@
         <v>31</v>
       </c>
       <c r="E577" s="98" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="F577" s="98" t="s">
         <v>228</v>
@@ -36760,7 +37161,7 @@
         <v>31</v>
       </c>
       <c r="E578" s="98" t="s">
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="F578" s="98" t="s">
         <v>228</v>
@@ -36775,12 +37176,12 @@
     <row r="579" spans="1:12" ht="27" customHeight="1">
       <c r="A579" s="92"/>
       <c r="B579" s="93"/>
-      <c r="C579" s="98"/>
+      <c r="C579" s="11"/>
       <c r="D579" s="99" t="s">
         <v>51</v>
       </c>
       <c r="E579" s="98" t="s">
-        <v>251</v>
+        <v>15</v>
       </c>
       <c r="F579" s="98" t="s">
         <v>228</v>
@@ -36800,7 +37201,7 @@
         <v>36</v>
       </c>
       <c r="E580" s="98" t="s">
-        <v>287</v>
+        <v>171</v>
       </c>
       <c r="F580" s="98" t="s">
         <v>228</v>
@@ -36813,111 +37214,312 @@
       <c r="L580" s="98"/>
     </row>
     <row r="581" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A581" s="5"/>
-      <c r="B581" s="36"/>
-      <c r="C581" s="37"/>
-      <c r="D581" s="38"/>
-      <c r="E581" s="37"/>
-      <c r="F581" s="37"/>
-      <c r="G581" s="37"/>
-      <c r="H581" s="37"/>
-      <c r="I581" s="39"/>
-      <c r="J581" s="37"/>
-      <c r="K581" s="37"/>
-      <c r="L581" s="37"/>
+      <c r="A581" s="92"/>
+      <c r="B581" s="93"/>
+      <c r="C581" s="98"/>
+      <c r="D581" s="99"/>
+      <c r="E581" s="98"/>
+      <c r="F581" s="98"/>
+      <c r="G581" s="98"/>
+      <c r="H581" s="98"/>
+      <c r="I581" s="99"/>
+      <c r="J581" s="98"/>
+      <c r="K581" s="98"/>
+      <c r="L581" s="98"/>
     </row>
     <row r="582" spans="1:12" ht="27" customHeight="1">
-      <c r="A582" s="100" t="s">
+      <c r="A582" s="92"/>
+      <c r="B582" s="97" t="s">
+        <v>86</v>
+      </c>
+      <c r="C582" s="98"/>
+      <c r="D582" s="99" t="s">
+        <v>21</v>
+      </c>
+      <c r="E582" s="98" t="s">
+        <v>281</v>
+      </c>
+      <c r="F582" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G582" s="98"/>
+      <c r="H582" s="98"/>
+      <c r="I582" s="99"/>
+      <c r="J582" s="98"/>
+      <c r="K582" s="98"/>
+      <c r="L582" s="98"/>
+    </row>
+    <row r="583" spans="1:12" ht="27" customHeight="1">
+      <c r="A583" s="92"/>
+      <c r="B583" s="93"/>
+      <c r="C583" s="98"/>
+      <c r="D583" s="99" t="s">
+        <v>24</v>
+      </c>
+      <c r="E583" s="98" t="s">
+        <v>289</v>
+      </c>
+      <c r="F583" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G583" s="98"/>
+      <c r="H583" s="98"/>
+      <c r="I583" s="99"/>
+      <c r="J583" s="98"/>
+      <c r="K583" s="98"/>
+      <c r="L583" s="98"/>
+    </row>
+    <row r="584" spans="1:12" ht="27" customHeight="1">
+      <c r="A584" s="92"/>
+      <c r="B584" s="93"/>
+      <c r="C584" s="98"/>
+      <c r="D584" s="99" t="s">
+        <v>24</v>
+      </c>
+      <c r="E584" s="98" t="s">
+        <v>290</v>
+      </c>
+      <c r="F584" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G584" s="98"/>
+      <c r="H584" s="98"/>
+      <c r="I584" s="99"/>
+      <c r="J584" s="98"/>
+      <c r="K584" s="98"/>
+      <c r="L584" s="98"/>
+    </row>
+    <row r="585" spans="1:12" ht="27" customHeight="1">
+      <c r="A585" s="92"/>
+      <c r="B585" s="93"/>
+      <c r="C585" s="98"/>
+      <c r="D585" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E585" s="98" t="s">
+        <v>282</v>
+      </c>
+      <c r="F585" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G585" s="98"/>
+      <c r="H585" s="98"/>
+      <c r="I585" s="99"/>
+      <c r="J585" s="98"/>
+      <c r="K585" s="98"/>
+      <c r="L585" s="98"/>
+    </row>
+    <row r="586" spans="1:12" ht="27" customHeight="1">
+      <c r="A586" s="92"/>
+      <c r="B586" s="93"/>
+      <c r="C586" s="98"/>
+      <c r="D586" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E586" s="98" t="s">
+        <v>219</v>
+      </c>
+      <c r="F586" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G586" s="98"/>
+      <c r="H586" s="98"/>
+      <c r="I586" s="99"/>
+      <c r="J586" s="98"/>
+      <c r="K586" s="98"/>
+      <c r="L586" s="98"/>
+    </row>
+    <row r="587" spans="1:12" ht="27" customHeight="1">
+      <c r="A587" s="92"/>
+      <c r="B587" s="93"/>
+      <c r="C587" s="98"/>
+      <c r="D587" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E587" s="98" t="s">
+        <v>226</v>
+      </c>
+      <c r="F587" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G587" s="98"/>
+      <c r="H587" s="98"/>
+      <c r="I587" s="99"/>
+      <c r="J587" s="98"/>
+      <c r="K587" s="98"/>
+      <c r="L587" s="98"/>
+    </row>
+    <row r="588" spans="1:12" ht="27" customHeight="1">
+      <c r="A588" s="92"/>
+      <c r="B588" s="93"/>
+      <c r="C588" s="98"/>
+      <c r="D588" s="99" t="s">
+        <v>31</v>
+      </c>
+      <c r="E588" s="98" t="s">
+        <v>280</v>
+      </c>
+      <c r="F588" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G588" s="98"/>
+      <c r="H588" s="98"/>
+      <c r="I588" s="99"/>
+      <c r="J588" s="98"/>
+      <c r="K588" s="98"/>
+      <c r="L588" s="98"/>
+    </row>
+    <row r="589" spans="1:12" ht="27" customHeight="1">
+      <c r="A589" s="92"/>
+      <c r="B589" s="93"/>
+      <c r="C589" s="98"/>
+      <c r="D589" s="99" t="s">
+        <v>31</v>
+      </c>
+      <c r="E589" s="98" t="s">
+        <v>171</v>
+      </c>
+      <c r="F589" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G589" s="98"/>
+      <c r="H589" s="98"/>
+      <c r="I589" s="99"/>
+      <c r="J589" s="98"/>
+      <c r="K589" s="98"/>
+      <c r="L589" s="98"/>
+    </row>
+    <row r="590" spans="1:12" ht="27" customHeight="1">
+      <c r="A590" s="92"/>
+      <c r="B590" s="93"/>
+      <c r="C590" s="98"/>
+      <c r="D590" s="99" t="s">
+        <v>51</v>
+      </c>
+      <c r="E590" s="98" t="s">
+        <v>251</v>
+      </c>
+      <c r="F590" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G590" s="98"/>
+      <c r="H590" s="98"/>
+      <c r="I590" s="99"/>
+      <c r="J590" s="98"/>
+      <c r="K590" s="98"/>
+      <c r="L590" s="98"/>
+    </row>
+    <row r="591" spans="1:12" ht="27" customHeight="1">
+      <c r="A591" s="92"/>
+      <c r="B591" s="93"/>
+      <c r="C591" s="98"/>
+      <c r="D591" s="99" t="s">
+        <v>36</v>
+      </c>
+      <c r="E591" s="98" t="s">
+        <v>287</v>
+      </c>
+      <c r="F591" s="98" t="s">
+        <v>228</v>
+      </c>
+      <c r="G591" s="98"/>
+      <c r="H591" s="98"/>
+      <c r="I591" s="99"/>
+      <c r="J591" s="98"/>
+      <c r="K591" s="98"/>
+      <c r="L591" s="98"/>
+    </row>
+    <row r="592" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A592" s="5"/>
+      <c r="B592" s="36"/>
+      <c r="C592" s="37"/>
+      <c r="D592" s="38"/>
+      <c r="E592" s="37"/>
+      <c r="F592" s="37"/>
+      <c r="G592" s="37"/>
+      <c r="H592" s="37"/>
+      <c r="I592" s="39"/>
+      <c r="J592" s="37"/>
+      <c r="K592" s="37"/>
+      <c r="L592" s="37"/>
+    </row>
+    <row r="593" spans="1:12" ht="27" customHeight="1">
+      <c r="A593" s="100" t="s">
         <v>291</v>
       </c>
-      <c r="B582" s="6"/>
-      <c r="C582" s="9"/>
-      <c r="D582" s="10"/>
-      <c r="E582" s="9"/>
-      <c r="F582" s="9"/>
-      <c r="G582" s="9"/>
-      <c r="H582" s="9"/>
-      <c r="I582" s="10"/>
-      <c r="J582" s="9"/>
-      <c r="K582" s="9"/>
-      <c r="L582" s="9"/>
-    </row>
-    <row r="583" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A583" s="100"/>
-      <c r="B583" s="6"/>
-      <c r="C583" s="9"/>
-      <c r="D583" s="10"/>
-      <c r="E583" s="9"/>
-      <c r="F583" s="9"/>
-      <c r="G583" s="9"/>
-      <c r="H583" s="9"/>
-      <c r="I583" s="10"/>
-      <c r="J583" s="9"/>
-      <c r="K583" s="9"/>
-      <c r="L583" s="9"/>
-    </row>
-    <row r="584" spans="1:12" ht="27" customHeight="1">
-      <c r="A584" s="100" t="s">
+      <c r="B593" s="6"/>
+      <c r="C593" s="9"/>
+      <c r="D593" s="10"/>
+      <c r="E593" s="9"/>
+      <c r="F593" s="9"/>
+      <c r="G593" s="9"/>
+      <c r="H593" s="9"/>
+      <c r="I593" s="10"/>
+      <c r="J593" s="9"/>
+      <c r="K593" s="9"/>
+      <c r="L593" s="9"/>
+    </row>
+    <row r="594" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A594" s="100"/>
+      <c r="B594" s="6"/>
+      <c r="C594" s="9"/>
+      <c r="D594" s="10"/>
+      <c r="E594" s="9"/>
+      <c r="F594" s="9"/>
+      <c r="G594" s="9"/>
+      <c r="H594" s="9"/>
+      <c r="I594" s="10"/>
+      <c r="J594" s="9"/>
+      <c r="K594" s="9"/>
+      <c r="L594" s="9"/>
+    </row>
+    <row r="595" spans="1:12" ht="27" customHeight="1">
+      <c r="A595" s="100" t="s">
         <v>292</v>
       </c>
-      <c r="B584" s="6"/>
-      <c r="C584" s="9"/>
-      <c r="D584" s="10"/>
-      <c r="E584" s="9"/>
-      <c r="F584" s="9"/>
-      <c r="G584" s="9"/>
-      <c r="H584" s="9"/>
-      <c r="I584" s="10"/>
-      <c r="J584" s="9"/>
-      <c r="K584" s="9"/>
-      <c r="L584" s="9"/>
-    </row>
-    <row r="585" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A585" s="100"/>
-      <c r="B585" s="6"/>
-      <c r="C585" s="9"/>
-      <c r="D585" s="10"/>
-      <c r="E585" s="9"/>
-      <c r="F585" s="9"/>
-      <c r="G585" s="9"/>
-      <c r="H585" s="9"/>
-      <c r="I585" s="10"/>
-      <c r="J585" s="9"/>
-      <c r="K585" s="9"/>
-      <c r="L585" s="9"/>
-    </row>
-    <row r="586" spans="1:12" ht="27" customHeight="1">
-      <c r="A586" s="100" t="s">
-        <v>293</v>
-      </c>
-      <c r="B586" s="6"/>
-      <c r="C586" s="9"/>
-      <c r="D586" s="10"/>
-      <c r="E586" s="9"/>
-      <c r="F586" s="9"/>
-      <c r="G586" s="9"/>
-      <c r="H586" s="9"/>
-      <c r="I586" s="10"/>
-      <c r="J586" s="9"/>
-      <c r="K586" s="9"/>
-      <c r="L586" s="9"/>
-    </row>
-    <row r="587" spans="1:12" ht="15.75" customHeight="1">
-      <c r="A587" s="5"/>
-      <c r="B587" s="6"/>
-      <c r="C587" s="9"/>
-      <c r="D587" s="10"/>
-      <c r="E587" s="9"/>
-      <c r="F587" s="9"/>
-      <c r="G587" s="9"/>
-      <c r="H587" s="9"/>
-      <c r="I587" s="10"/>
-      <c r="J587" s="9"/>
-      <c r="K587" s="9"/>
-      <c r="L587" s="9"/>
+      <c r="B595" s="6"/>
+      <c r="C595" s="9"/>
+      <c r="D595" s="10"/>
+      <c r="E595" s="9"/>
+      <c r="F595" s="9"/>
+      <c r="G595" s="9"/>
+      <c r="H595" s="9"/>
+      <c r="I595" s="10"/>
+      <c r="J595" s="9"/>
+      <c r="K595" s="9"/>
+      <c r="L595" s="9"/>
+    </row>
+    <row r="596" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A596" s="100"/>
+      <c r="B596" s="6"/>
+      <c r="C596" s="9"/>
+      <c r="D596" s="10"/>
+      <c r="E596" s="9"/>
+      <c r="F596" s="9"/>
+      <c r="G596" s="9"/>
+      <c r="H596" s="9"/>
+      <c r="I596" s="10"/>
+      <c r="J596" s="9"/>
+      <c r="K596" s="9"/>
+      <c r="L596" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="A114:A115"/>
+    <mergeCell ref="A125:A126"/>
+    <mergeCell ref="A136:A137"/>
+    <mergeCell ref="A147:A148"/>
+    <mergeCell ref="A162:A163"/>
+    <mergeCell ref="A173:A174"/>
+    <mergeCell ref="A184:A185"/>
+    <mergeCell ref="A231:A232"/>
+    <mergeCell ref="A242:A243"/>
+    <mergeCell ref="A342:A343"/>
     <mergeCell ref="B311:B312"/>
     <mergeCell ref="B321:B322"/>
     <mergeCell ref="B332:B333"/>
@@ -36931,21 +37533,6 @@
     <mergeCell ref="A384:A385"/>
     <mergeCell ref="A393:A394"/>
     <mergeCell ref="A496:A497"/>
-    <mergeCell ref="A173:A174"/>
-    <mergeCell ref="A184:A185"/>
-    <mergeCell ref="A231:A232"/>
-    <mergeCell ref="A242:A243"/>
-    <mergeCell ref="A342:A343"/>
-    <mergeCell ref="A114:A115"/>
-    <mergeCell ref="A125:A126"/>
-    <mergeCell ref="A136:A137"/>
-    <mergeCell ref="A147:A148"/>
-    <mergeCell ref="A162:A163"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A68:A69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>